<commit_message>
Clean colnames when loading in df, preventing bugs downstream
</commit_message>
<xml_diff>
--- a/example_data/metadata.xlsx
+++ b/example_data/metadata.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\m.leeuwerik\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{431875C0-A5D5-4C09-B47A-89AE82DC4457}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26ACC3F0-16A2-4CF0-8953-F6CFA7DA9C80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Rhodes_metadata" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2267" uniqueCount="273">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2268" uniqueCount="274">
   <si>
     <t>ARAF001</t>
   </si>
@@ -844,6 +845,9 @@
   </si>
   <si>
     <t>Clade</t>
+  </si>
+  <si>
+    <t>`Empty` sheet 2</t>
   </si>
 </sst>
 </file>
@@ -11332,4 +11336,22 @@
     <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3953F869-36B8-4C2E-B964-F9A75DCFFBB7}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>273</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>